<commit_message>
synthetic data revised patient_id columns for NHI validation
</commit_message>
<xml_diff>
--- a/inst/extdata/a3_2025.xlsx
+++ b/inst/extdata/a3_2025.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -52,10 +51,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -557,10 +557,10 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SPD001</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
+          <t>SPD0001</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
         <v>29897</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -594,7 +594,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="3" t="n">
         <v>43878</v>
       </c>
       <c r="K2" t="inlineStr">
@@ -602,7 +602,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L2" s="2" t="n">
+      <c r="L2" s="3" t="n">
         <v>43905</v>
       </c>
       <c r="O2" t="inlineStr">
@@ -614,10 +614,10 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SPD002</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
+          <t>SPD0002</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
         <v>17104</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -651,7 +651,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="3" t="n">
         <v>44011</v>
       </c>
       <c r="K3" t="inlineStr">
@@ -659,7 +659,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L3" s="2" t="n">
+      <c r="L3" s="3" t="n">
         <v>44034</v>
       </c>
       <c r="O3" t="inlineStr">
@@ -671,10 +671,10 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SPD003</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
+          <t>SPD0003</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
         <v>25389</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -708,7 +708,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="3" t="n">
         <v>44125</v>
       </c>
       <c r="K4" t="inlineStr">
@@ -716,7 +716,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="L4" s="3" t="n">
         <v>44145</v>
       </c>
       <c r="O4" t="inlineStr">
@@ -728,10 +728,10 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SPD004</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
+          <t>SPD0004</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
         <v>26813</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -765,7 +765,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="3" t="n">
         <v>44180</v>
       </c>
       <c r="K5" t="inlineStr">
@@ -773,7 +773,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L5" s="2" t="n">
+      <c r="L5" s="3" t="n">
         <v>44204</v>
       </c>
       <c r="O5" t="inlineStr">
@@ -785,10 +785,10 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SPD005</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
+          <t>SPD0005</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
         <v>24518</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -822,7 +822,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="3" t="n">
         <v>44264</v>
       </c>
       <c r="K6" t="inlineStr">
@@ -830,7 +830,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L6" s="2" t="n">
+      <c r="L6" s="3" t="n">
         <v>44280</v>
       </c>
       <c r="O6" t="inlineStr">
@@ -842,10 +842,10 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SPD006</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
+          <t>SPD0006</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
         <v>16516</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -879,7 +879,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="3" t="n">
         <v>44302</v>
       </c>
       <c r="K7" t="inlineStr">
@@ -887,7 +887,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L7" s="2" t="n">
+      <c r="L7" s="3" t="n">
         <v>44330</v>
       </c>
       <c r="O7" t="inlineStr">
@@ -899,10 +899,10 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SPD007</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
+          <t>SPD0007</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
         <v>27093</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -936,7 +936,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="3" t="n">
         <v>44399</v>
       </c>
       <c r="K8" t="inlineStr">
@@ -944,7 +944,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L8" s="2" t="n">
+      <c r="L8" s="3" t="n">
         <v>44407</v>
       </c>
       <c r="O8" t="inlineStr">
@@ -956,10 +956,10 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SPD008</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
+          <t>SPD0008</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
         <v>20811</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -993,7 +993,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="3" t="n">
         <v>44430</v>
       </c>
       <c r="K9" t="inlineStr">
@@ -1001,7 +1001,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="L9" s="3" t="n">
         <v>44457</v>
       </c>
       <c r="O9" t="inlineStr">
@@ -1013,10 +1013,10 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SPD009</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
+          <t>SPD0009</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
         <v>30401</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -1050,7 +1050,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="J10" s="3" t="n">
         <v>44482</v>
       </c>
       <c r="K10" t="inlineStr">
@@ -1058,7 +1058,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L10" s="2" t="n">
+      <c r="L10" s="3" t="n">
         <v>44505</v>
       </c>
       <c r="O10" t="inlineStr">
@@ -1070,10 +1070,10 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SPD010</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
+          <t>SPD0010</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
         <v>16692</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -1107,7 +1107,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="3" t="n">
         <v>44558</v>
       </c>
       <c r="K11" t="inlineStr">
@@ -1115,7 +1115,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L11" s="2" t="n">
+      <c r="L11" s="3" t="n">
         <v>44573</v>
       </c>
       <c r="O11" t="inlineStr">
@@ -1127,10 +1127,10 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SPD011</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
+          <t>SPD0011</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
         <v>21885</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -1164,7 +1164,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="3" t="n">
         <v>44599</v>
       </c>
       <c r="K12" t="inlineStr">
@@ -1172,7 +1172,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L12" s="2" t="n">
+      <c r="L12" s="3" t="n">
         <v>44620</v>
       </c>
       <c r="O12" t="inlineStr">
@@ -1184,10 +1184,10 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SPD012</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
+          <t>SPD0012</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
         <v>21475</v>
       </c>
       <c r="C13" t="inlineStr">
@@ -1221,7 +1221,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J13" s="2" t="n">
+      <c r="J13" s="3" t="n">
         <v>44648</v>
       </c>
       <c r="K13" t="inlineStr">
@@ -1229,7 +1229,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L13" s="2" t="n">
+      <c r="L13" s="3" t="n">
         <v>44666</v>
       </c>
       <c r="O13" t="inlineStr">
@@ -1241,10 +1241,10 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SPD013</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
+          <t>SPD0013</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
         <v>31999</v>
       </c>
       <c r="C14" t="inlineStr">
@@ -1278,7 +1278,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="J14" s="3" t="n">
         <v>44701</v>
       </c>
       <c r="K14" t="inlineStr">
@@ -1286,7 +1286,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L14" s="2" t="n">
+      <c r="L14" s="3" t="n">
         <v>44715</v>
       </c>
       <c r="O14" t="inlineStr">
@@ -1298,10 +1298,10 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SPD014</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
+          <t>SPD0014</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
         <v>29152</v>
       </c>
       <c r="C15" t="inlineStr">
@@ -1335,7 +1335,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="J15" s="3" t="n">
         <v>44750</v>
       </c>
       <c r="K15" t="inlineStr">
@@ -1343,7 +1343,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L15" s="2" t="n">
+      <c r="L15" s="3" t="n">
         <v>44762</v>
       </c>
       <c r="O15" t="inlineStr">
@@ -1355,10 +1355,10 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SPD015</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
+          <t>SPD0015</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
         <v>33610</v>
       </c>
       <c r="C16" t="inlineStr">
@@ -1392,7 +1392,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="J16" s="3" t="n">
         <v>44789</v>
       </c>
       <c r="K16" t="inlineStr">
@@ -1400,7 +1400,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L16" s="2" t="n">
+      <c r="L16" s="3" t="n">
         <v>44812</v>
       </c>
       <c r="O16" t="inlineStr">
@@ -1412,10 +1412,10 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SPD016</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
+          <t>SPD0016</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
         <v>18629</v>
       </c>
       <c r="C17" t="inlineStr">
@@ -1449,7 +1449,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J17" s="2" t="n">
+      <c r="J17" s="3" t="n">
         <v>44851</v>
       </c>
       <c r="K17" t="inlineStr">
@@ -1457,7 +1457,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L17" s="2" t="n">
+      <c r="L17" s="3" t="n">
         <v>44859</v>
       </c>
       <c r="O17" t="inlineStr">
@@ -1469,10 +1469,10 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SPD017</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
+          <t>SPD0017</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
         <v>24116</v>
       </c>
       <c r="C18" t="inlineStr">
@@ -1506,7 +1506,7 @@
           <t>Type 1</t>
         </is>
       </c>
-      <c r="J18" s="2" t="n">
+      <c r="J18" s="3" t="n">
         <v>44885</v>
       </c>
       <c r="K18" t="inlineStr">
@@ -1514,7 +1514,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L18" s="2" t="n">
+      <c r="L18" s="3" t="n">
         <v>44905</v>
       </c>
       <c r="O18" t="inlineStr">
@@ -1526,10 +1526,10 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SPD018</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
+          <t>SPD0018</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
         <v>21617</v>
       </c>
       <c r="C19" t="inlineStr">
@@ -1563,7 +1563,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J19" s="2" t="n">
+      <c r="J19" s="3" t="n">
         <v>44927</v>
       </c>
       <c r="K19" t="inlineStr">
@@ -1571,7 +1571,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L19" s="2" t="n">
+      <c r="L19" s="3" t="n">
         <v>44944</v>
       </c>
       <c r="O19" t="inlineStr">
@@ -1583,10 +1583,10 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SPD019</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
+          <t>SPD0019</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
         <v>33900</v>
       </c>
       <c r="C20" t="inlineStr">
@@ -1620,7 +1620,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J20" s="2" t="n">
+      <c r="J20" s="3" t="n">
         <v>44966</v>
       </c>
       <c r="K20" t="inlineStr">
@@ -1628,7 +1628,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L20" s="2" t="n">
+      <c r="L20" s="3" t="n">
         <v>44990</v>
       </c>
       <c r="O20" t="inlineStr">
@@ -1640,10 +1640,10 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SPD020</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
+          <t>SPD0020</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
         <v>23455</v>
       </c>
       <c r="C21" t="inlineStr">
@@ -1677,7 +1677,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J21" s="2" t="n">
+      <c r="J21" s="3" t="n">
         <v>45030</v>
       </c>
       <c r="K21" t="inlineStr">
@@ -1685,7 +1685,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L21" s="2" t="n">
+      <c r="L21" s="3" t="n">
         <v>45038</v>
       </c>
       <c r="O21" t="inlineStr">
@@ -1697,10 +1697,10 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SPD021</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n">
+          <t>SPD0021</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
         <v>33003</v>
       </c>
       <c r="C22" t="inlineStr">
@@ -1734,7 +1734,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J22" s="2" t="n">
+      <c r="J22" s="3" t="n">
         <v>45060</v>
       </c>
       <c r="K22" t="inlineStr">
@@ -1742,7 +1742,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L22" s="2" t="n">
+      <c r="L22" s="3" t="n">
         <v>45076</v>
       </c>
       <c r="O22" t="inlineStr">
@@ -1754,10 +1754,10 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SPD022</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="n">
+          <t>SPD0022</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
         <v>28712</v>
       </c>
       <c r="C23" t="inlineStr">
@@ -1791,7 +1791,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J23" s="2" t="n">
+      <c r="J23" s="3" t="n">
         <v>45113</v>
       </c>
       <c r="K23" t="inlineStr">
@@ -1799,7 +1799,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L23" s="2" t="n">
+      <c r="L23" s="3" t="n">
         <v>45122</v>
       </c>
       <c r="O23" t="inlineStr">
@@ -1811,10 +1811,10 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SPD023</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="n">
+          <t>SPD0023</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
         <v>18848</v>
       </c>
       <c r="C24" t="inlineStr">
@@ -1848,7 +1848,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J24" s="2" t="n">
+      <c r="J24" s="3" t="n">
         <v>45141</v>
       </c>
       <c r="K24" t="inlineStr">
@@ -1856,7 +1856,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L24" s="2" t="n">
+      <c r="L24" s="3" t="n">
         <v>45166</v>
       </c>
       <c r="O24" t="inlineStr">
@@ -1868,10 +1868,10 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SPD024</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
+          <t>SPD0024</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
         <v>31917</v>
       </c>
       <c r="C25" t="inlineStr">
@@ -1905,7 +1905,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J25" s="2" t="n">
+      <c r="J25" s="3" t="n">
         <v>45200</v>
       </c>
       <c r="K25" t="inlineStr">
@@ -1913,7 +1913,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L25" s="2" t="n">
+      <c r="L25" s="3" t="n">
         <v>45209</v>
       </c>
       <c r="O25" t="inlineStr">
@@ -1925,10 +1925,10 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SPD025</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n">
+          <t>SPD0025</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
         <v>20202</v>
       </c>
       <c r="C26" t="inlineStr">
@@ -1962,7 +1962,7 @@
           <t>Type 1</t>
         </is>
       </c>
-      <c r="J26" s="2" t="n">
+      <c r="J26" s="3" t="n">
         <v>45234</v>
       </c>
       <c r="K26" t="inlineStr">
@@ -1970,7 +1970,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L26" s="2" t="n">
+      <c r="L26" s="3" t="n">
         <v>45250</v>
       </c>
       <c r="O26" t="inlineStr">
@@ -1982,10 +1982,10 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SPD026</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
+          <t>SPD0026</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
         <v>28097</v>
       </c>
       <c r="C27" t="inlineStr">
@@ -2019,7 +2019,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J27" s="2" t="n">
+      <c r="J27" s="3" t="n">
         <v>45284</v>
       </c>
       <c r="K27" t="inlineStr">
@@ -2027,7 +2027,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L27" s="2" t="n">
+      <c r="L27" s="3" t="n">
         <v>45299</v>
       </c>
       <c r="O27" t="inlineStr">
@@ -2039,10 +2039,10 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SPD027</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n">
+          <t>SPD0027</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
         <v>34369</v>
       </c>
       <c r="C28" t="inlineStr">
@@ -2076,7 +2076,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J28" s="2" t="n">
+      <c r="J28" s="3" t="n">
         <v>45328</v>
       </c>
       <c r="K28" t="inlineStr">
@@ -2084,7 +2084,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L28" s="2" t="n">
+      <c r="L28" s="3" t="n">
         <v>45336</v>
       </c>
       <c r="O28" t="inlineStr">
@@ -2096,10 +2096,10 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SPD028</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="n">
+          <t>SPD0028</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
         <v>31227</v>
       </c>
       <c r="C29" t="inlineStr">
@@ -2133,7 +2133,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J29" s="2" t="n">
+      <c r="J29" s="3" t="n">
         <v>45366</v>
       </c>
       <c r="K29" t="inlineStr">
@@ -2141,7 +2141,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L29" s="2" t="n">
+      <c r="L29" s="3" t="n">
         <v>45373</v>
       </c>
       <c r="O29" t="inlineStr">
@@ -2153,10 +2153,10 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SPD029</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="n">
+          <t>SPD0029</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
         <v>32264</v>
       </c>
       <c r="C30" t="inlineStr">
@@ -2190,7 +2190,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J30" s="2" t="n">
+      <c r="J30" s="3" t="n">
         <v>45404</v>
       </c>
       <c r="K30" t="inlineStr">
@@ -2198,7 +2198,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L30" s="2" t="n">
+      <c r="L30" s="3" t="n">
         <v>45412</v>
       </c>
       <c r="O30" t="inlineStr">
@@ -2210,10 +2210,10 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SPD030</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n">
+          <t>SPD0030</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
         <v>34018</v>
       </c>
       <c r="C31" t="inlineStr">
@@ -2247,7 +2247,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J31" s="2" t="n">
+      <c r="J31" s="3" t="n">
         <v>45418</v>
       </c>
       <c r="K31" t="inlineStr">
@@ -2255,7 +2255,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L31" s="2" t="n">
+      <c r="L31" s="3" t="n">
         <v>45430</v>
       </c>
       <c r="O31" t="inlineStr">
@@ -2267,10 +2267,10 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SPD031</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n">
+          <t>SPD0031</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
         <v>33840</v>
       </c>
       <c r="C32" t="inlineStr">
@@ -2304,7 +2304,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J32" s="2" t="n">
+      <c r="J32" s="3" t="n">
         <v>45453</v>
       </c>
       <c r="K32" t="inlineStr">
@@ -2312,7 +2312,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L32" s="2" t="n">
+      <c r="L32" s="3" t="n">
         <v>45468</v>
       </c>
       <c r="O32" t="inlineStr">
@@ -2324,10 +2324,10 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SPD032</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="n">
+          <t>SPD0032</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
         <v>33031</v>
       </c>
       <c r="C33" t="inlineStr">
@@ -2361,7 +2361,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J33" s="2" t="n">
+      <c r="J33" s="3" t="n">
         <v>45481</v>
       </c>
       <c r="K33" t="inlineStr">
@@ -2369,7 +2369,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L33" s="2" t="n">
+      <c r="L33" s="3" t="n">
         <v>45488</v>
       </c>
       <c r="O33" t="inlineStr">
@@ -2381,10 +2381,10 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SPD033</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="n">
+          <t>SPD0033</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
         <v>32490</v>
       </c>
       <c r="C34" t="inlineStr">
@@ -2418,7 +2418,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J34" s="2" t="n">
+      <c r="J34" s="3" t="n">
         <v>45499</v>
       </c>
       <c r="K34" t="inlineStr">
@@ -2426,7 +2426,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L34" s="2" t="n">
+      <c r="L34" s="3" t="n">
         <v>45514</v>
       </c>
       <c r="O34" t="inlineStr">
@@ -2438,10 +2438,10 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SPD034</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="n">
+          <t>SPD0034</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
         <v>22624</v>
       </c>
       <c r="C35" t="inlineStr">
@@ -2475,7 +2475,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J35" s="2" t="n">
+      <c r="J35" s="3" t="n">
         <v>45515</v>
       </c>
       <c r="K35" t="inlineStr">
@@ -2483,7 +2483,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L35" s="2" t="n">
+      <c r="L35" s="3" t="n">
         <v>45540</v>
       </c>
       <c r="O35" t="inlineStr">
@@ -2495,10 +2495,10 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SPD035</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="n">
+          <t>SPD0035</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
         <v>27747</v>
       </c>
       <c r="C36" t="inlineStr">
@@ -2532,7 +2532,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J36" s="2" t="n">
+      <c r="J36" s="3" t="n">
         <v>45549</v>
       </c>
       <c r="K36" t="inlineStr">
@@ -2540,7 +2540,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L36" s="2" t="n">
+      <c r="L36" s="3" t="n">
         <v>45566</v>
       </c>
       <c r="O36" t="inlineStr">
@@ -2552,10 +2552,10 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SPD036</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="n">
+          <t>SPD0036</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
         <v>27716</v>
       </c>
       <c r="C37" t="inlineStr">
@@ -2589,7 +2589,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J37" s="2" t="n">
+      <c r="J37" s="3" t="n">
         <v>45568</v>
       </c>
       <c r="K37" t="inlineStr">
@@ -2597,7 +2597,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L37" s="2" t="n">
+      <c r="L37" s="3" t="n">
         <v>45587</v>
       </c>
       <c r="O37" t="inlineStr">
@@ -2609,10 +2609,10 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SPD037</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="n">
+          <t>SPD0037</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
         <v>17385</v>
       </c>
       <c r="C38" t="inlineStr">
@@ -2646,7 +2646,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J38" s="2" t="n">
+      <c r="J38" s="3" t="n">
         <v>45583</v>
       </c>
       <c r="K38" t="inlineStr">
@@ -2654,7 +2654,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L38" s="2" t="n">
+      <c r="L38" s="3" t="n">
         <v>45604</v>
       </c>
       <c r="O38" t="inlineStr">
@@ -2666,10 +2666,10 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SPD038</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="n">
+          <t>SPD0038</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
         <v>34141</v>
       </c>
       <c r="C39" t="inlineStr">
@@ -2703,7 +2703,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J39" s="2" t="n">
+      <c r="J39" s="3" t="n">
         <v>45607</v>
       </c>
       <c r="K39" t="inlineStr">
@@ -2711,7 +2711,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L39" s="2" t="n">
+      <c r="L39" s="3" t="n">
         <v>45621</v>
       </c>
       <c r="O39" t="inlineStr">
@@ -2723,10 +2723,10 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SPD039</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="n">
+          <t>SPD0039</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
         <v>31541</v>
       </c>
       <c r="C40" t="inlineStr">
@@ -2760,7 +2760,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J40" s="2" t="n">
+      <c r="J40" s="3" t="n">
         <v>45618</v>
       </c>
       <c r="K40" t="inlineStr">
@@ -2768,7 +2768,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L40" s="2" t="n">
+      <c r="L40" s="3" t="n">
         <v>45631</v>
       </c>
       <c r="O40" t="inlineStr">
@@ -2780,10 +2780,10 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SPD040</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="n">
+          <t>SPD0040</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
         <v>32182</v>
       </c>
       <c r="C41" t="inlineStr">
@@ -2817,7 +2817,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J41" s="2" t="n">
+      <c r="J41" s="3" t="n">
         <v>45621</v>
       </c>
       <c r="K41" t="inlineStr">
@@ -2825,7 +2825,7 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L41" s="2" t="n">
+      <c r="L41" s="3" t="n">
         <v>45644</v>
       </c>
       <c r="O41" t="inlineStr">
@@ -2837,10 +2837,10 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SPD041</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="n">
+          <t>SPD0041</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
         <v>21978</v>
       </c>
       <c r="C42" t="inlineStr">
@@ -2874,7 +2874,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J42" s="2" t="n">
+      <c r="J42" s="3" t="n">
         <v>45658</v>
       </c>
       <c r="K42" t="inlineStr">
@@ -2882,7 +2882,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L42" s="2" t="n">
+      <c r="L42" s="3" t="n">
         <v>45672</v>
       </c>
       <c r="O42" t="inlineStr">
@@ -2894,10 +2894,10 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SPD042</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="n">
+          <t>SPD0042</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
         <v>24372</v>
       </c>
       <c r="C43" t="inlineStr">
@@ -2931,7 +2931,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J43" s="2" t="n">
+      <c r="J43" s="3" t="n">
         <v>45679</v>
       </c>
       <c r="K43" t="inlineStr">
@@ -2939,7 +2939,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L43" s="2" t="n">
+      <c r="L43" s="3" t="n">
         <v>45698</v>
       </c>
       <c r="O43" t="inlineStr">
@@ -2951,10 +2951,10 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SPD043</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="n">
+          <t>SPD0043</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
         <v>25256</v>
       </c>
       <c r="C44" t="inlineStr">
@@ -2988,7 +2988,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J44" s="2" t="n">
+      <c r="J44" s="3" t="n">
         <v>45708</v>
       </c>
       <c r="K44" t="inlineStr">
@@ -2996,7 +2996,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L44" s="2" t="n">
+      <c r="L44" s="3" t="n">
         <v>45721</v>
       </c>
       <c r="O44" t="inlineStr">
@@ -3008,10 +3008,10 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SPD044</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="n">
+          <t>SPD0044</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
         <v>23656</v>
       </c>
       <c r="C45" t="inlineStr">
@@ -3045,7 +3045,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J45" s="2" t="n">
+      <c r="J45" s="3" t="n">
         <v>45730</v>
       </c>
       <c r="K45" t="inlineStr">
@@ -3053,7 +3053,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L45" s="2" t="n">
+      <c r="L45" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="O45" t="inlineStr">
@@ -3065,10 +3065,10 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SPD045</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="n">
+          <t>SPD0045</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
         <v>29677</v>
       </c>
       <c r="C46" t="inlineStr">
@@ -3102,7 +3102,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J46" s="2" t="n">
+      <c r="J46" s="3" t="n">
         <v>45771</v>
       </c>
       <c r="K46" t="inlineStr">
@@ -3110,7 +3110,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L46" s="2" t="n">
+      <c r="L46" s="3" t="n">
         <v>45789</v>
       </c>
       <c r="O46" t="inlineStr">
@@ -3122,10 +3122,10 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SPD046</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="n">
+          <t>SPD0046</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
         <v>25862</v>
       </c>
       <c r="C47" t="inlineStr">
@@ -3159,7 +3159,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J47" s="2" t="n">
+      <c r="J47" s="3" t="n">
         <v>45814</v>
       </c>
       <c r="K47" t="inlineStr">
@@ -3167,7 +3167,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L47" s="2" t="n">
+      <c r="L47" s="3" t="n">
         <v>45828</v>
       </c>
       <c r="O47" t="inlineStr">
@@ -3179,10 +3179,10 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SPD047</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="n">
+          <t>SPD0047</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
         <v>26091</v>
       </c>
       <c r="C48" t="inlineStr">
@@ -3216,7 +3216,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J48" s="2" t="n">
+      <c r="J48" s="3" t="n">
         <v>45840</v>
       </c>
       <c r="K48" t="inlineStr">
@@ -3224,7 +3224,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L48" s="2" t="n">
+      <c r="L48" s="3" t="n">
         <v>45853</v>
       </c>
       <c r="O48" t="inlineStr">
@@ -3236,10 +3236,10 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SPD048</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="n">
+          <t>SPD0048</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
         <v>34041</v>
       </c>
       <c r="C49" t="inlineStr">
@@ -3273,7 +3273,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J49" s="2" t="n">
+      <c r="J49" s="3" t="n">
         <v>45882</v>
       </c>
       <c r="K49" t="inlineStr">
@@ -3281,7 +3281,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L49" s="2" t="n">
+      <c r="L49" s="3" t="n">
         <v>45894</v>
       </c>
       <c r="O49" t="inlineStr">
@@ -3293,10 +3293,10 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SPD049</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="n">
+          <t>SPD0049</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
         <v>26457</v>
       </c>
       <c r="C50" t="inlineStr">
@@ -3330,7 +3330,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J50" s="2" t="n">
+      <c r="J50" s="3" t="n">
         <v>45894</v>
       </c>
       <c r="K50" t="inlineStr">
@@ -3338,7 +3338,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L50" s="2" t="n">
+      <c r="L50" s="3" t="n">
         <v>45910</v>
       </c>
       <c r="O50" t="inlineStr">
@@ -3350,10 +3350,10 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SPD050</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="n">
+          <t>SPD0050</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
         <v>26263</v>
       </c>
       <c r="C51" t="inlineStr">
@@ -3387,7 +3387,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J51" s="2" t="n">
+      <c r="J51" s="3" t="n">
         <v>45948</v>
       </c>
       <c r="K51" t="inlineStr">
@@ -3395,7 +3395,7 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L51" s="2" t="n">
+      <c r="L51" s="3" t="n">
         <v>45964</v>
       </c>
       <c r="O51" t="inlineStr">
@@ -3407,10 +3407,10 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SPD051</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="n">
+          <t>SPD0051</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
         <v>20426</v>
       </c>
       <c r="C52" t="inlineStr">
@@ -3444,7 +3444,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J52" s="2" t="n">
+      <c r="J52" s="3" t="n">
         <v>44675</v>
       </c>
       <c r="K52" t="inlineStr">
@@ -3452,10 +3452,10 @@
           <t>Percutaneous</t>
         </is>
       </c>
-      <c r="L52" s="2" t="n">
+      <c r="L52" s="3" t="n">
         <v>44691</v>
       </c>
-      <c r="M52" s="2" t="n">
+      <c r="M52" s="3" t="n">
         <v>45703</v>
       </c>
       <c r="N52" t="inlineStr">
@@ -3468,7 +3468,7 @@
           <t>CAPD</t>
         </is>
       </c>
-      <c r="S52" s="2" t="n">
+      <c r="S52" s="3" t="n">
         <v>45703</v>
       </c>
       <c r="T52" t="inlineStr">
@@ -3480,10 +3480,10 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SPD052</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="n">
+          <t>SPD0052</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
         <v>23352</v>
       </c>
       <c r="C53" t="inlineStr">
@@ -3517,7 +3517,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J53" s="2" t="n">
+      <c r="J53" s="3" t="n">
         <v>44981</v>
       </c>
       <c r="K53" t="inlineStr">
@@ -3525,10 +3525,10 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L53" s="2" t="n">
+      <c r="L53" s="3" t="n">
         <v>45003</v>
       </c>
-      <c r="M53" s="2" t="n">
+      <c r="M53" s="3" t="n">
         <v>45838</v>
       </c>
       <c r="N53" t="inlineStr">
@@ -3541,7 +3541,7 @@
           <t>APD</t>
         </is>
       </c>
-      <c r="S53" s="2" t="n">
+      <c r="S53" s="3" t="n">
         <v>45838</v>
       </c>
       <c r="T53" t="inlineStr">
@@ -3553,10 +3553,10 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SPD053</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="n">
+          <t>SPD0053</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
         <v>26112</v>
       </c>
       <c r="C54" t="inlineStr">
@@ -3590,7 +3590,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J54" s="2" t="n">
+      <c r="J54" s="3" t="n">
         <v>44408</v>
       </c>
       <c r="K54" t="inlineStr">
@@ -3598,10 +3598,10 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L54" s="2" t="n">
+      <c r="L54" s="3" t="n">
         <v>44430</v>
       </c>
-      <c r="M54" s="2" t="n">
+      <c r="M54" s="3" t="n">
         <v>45950</v>
       </c>
       <c r="N54" t="inlineStr">
@@ -3614,7 +3614,7 @@
           <t>APD</t>
         </is>
       </c>
-      <c r="S54" s="2" t="n">
+      <c r="S54" s="3" t="n">
         <v>45950</v>
       </c>
       <c r="T54" t="inlineStr">
@@ -3626,10 +3626,10 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SPD054</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="n">
+          <t>SPD0054</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
         <v>22822</v>
       </c>
       <c r="C55" t="inlineStr">
@@ -3663,7 +3663,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J55" s="2" t="n">
+      <c r="J55" s="3" t="n">
         <v>45155</v>
       </c>
       <c r="K55" t="inlineStr">
@@ -3671,10 +3671,10 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L55" s="2" t="n">
+      <c r="L55" s="3" t="n">
         <v>45174</v>
       </c>
-      <c r="M55" s="2" t="n">
+      <c r="M55" s="3" t="n">
         <v>45726</v>
       </c>
       <c r="N55" t="inlineStr">
@@ -3687,17 +3687,17 @@
           <t>APD</t>
         </is>
       </c>
-      <c r="U55" s="2" t="n">
+      <c r="U55" s="3" t="n">
         <v>45726</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SPD055</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="n">
+          <t>SPD0055</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
         <v>22704</v>
       </c>
       <c r="C56" t="inlineStr">
@@ -3731,7 +3731,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J56" s="2" t="n">
+      <c r="J56" s="3" t="n">
         <v>44857</v>
       </c>
       <c r="K56" t="inlineStr">
@@ -3739,10 +3739,10 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L56" s="2" t="n">
+      <c r="L56" s="3" t="n">
         <v>44880</v>
       </c>
-      <c r="M56" s="2" t="n">
+      <c r="M56" s="3" t="n">
         <v>45860</v>
       </c>
       <c r="N56" t="inlineStr">
@@ -3755,17 +3755,17 @@
           <t>APD</t>
         </is>
       </c>
-      <c r="U56" s="2" t="n">
+      <c r="U56" s="3" t="n">
         <v>45860</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SPD056</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="n">
+          <t>SPD0056</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
         <v>26015</v>
       </c>
       <c r="C57" t="inlineStr">
@@ -3799,7 +3799,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J57" s="2" t="n">
+      <c r="J57" s="3" t="n">
         <v>45297</v>
       </c>
       <c r="K57" t="inlineStr">
@@ -3807,10 +3807,10 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L57" s="2" t="n">
+      <c r="L57" s="3" t="n">
         <v>45311</v>
       </c>
-      <c r="M57" s="2" t="n">
+      <c r="M57" s="3" t="n">
         <v>45976</v>
       </c>
       <c r="N57" t="inlineStr">
@@ -3823,17 +3823,17 @@
           <t>CAPD</t>
         </is>
       </c>
-      <c r="U57" s="2" t="n">
+      <c r="U57" s="3" t="n">
         <v>45976</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SPD057</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="n">
+          <t>SPD0057</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
         <v>31669</v>
       </c>
       <c r="C58" t="inlineStr">
@@ -3867,7 +3867,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J58" s="2" t="n">
+      <c r="J58" s="3" t="n">
         <v>45073</v>
       </c>
       <c r="K58" t="inlineStr">
@@ -3875,10 +3875,10 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L58" s="2" t="n">
+      <c r="L58" s="3" t="n">
         <v>45089</v>
       </c>
-      <c r="M58" s="2" t="n">
+      <c r="M58" s="3" t="n">
         <v>45772</v>
       </c>
       <c r="N58" t="inlineStr">
@@ -3901,17 +3901,17 @@
           <t>Ultrafiltration failure</t>
         </is>
       </c>
-      <c r="R58" s="2" t="n">
+      <c r="R58" s="3" t="n">
         <v>45772</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SPD058</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="n">
+          <t>SPD0058</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="n">
         <v>27207</v>
       </c>
       <c r="C59" t="inlineStr">
@@ -3945,7 +3945,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="J59" s="2" t="n">
+      <c r="J59" s="3" t="n">
         <v>44780</v>
       </c>
       <c r="K59" t="inlineStr">
@@ -3953,10 +3953,10 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L59" s="2" t="n">
+      <c r="L59" s="3" t="n">
         <v>44803</v>
       </c>
-      <c r="M59" s="2" t="n">
+      <c r="M59" s="3" t="n">
         <v>45905</v>
       </c>
       <c r="N59" t="inlineStr">
@@ -3979,17 +3979,17 @@
           <t>Inadequate dialysis</t>
         </is>
       </c>
-      <c r="R59" s="2" t="n">
+      <c r="R59" s="3" t="n">
         <v>45905</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SPD059</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="n">
+          <t>SPD0059</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="n">
         <v>22922</v>
       </c>
       <c r="C60" t="inlineStr">
@@ -4023,7 +4023,7 @@
           <t>Type 2</t>
         </is>
       </c>
-      <c r="J60" s="2" t="n">
+      <c r="J60" s="3" t="n">
         <v>45314</v>
       </c>
       <c r="K60" t="inlineStr">
@@ -4031,10 +4031,10 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L60" s="2" t="n">
+      <c r="L60" s="3" t="n">
         <v>45330</v>
       </c>
-      <c r="M60" s="2" t="n">
+      <c r="M60" s="3" t="n">
         <v>45807</v>
       </c>
       <c r="N60" t="inlineStr">
@@ -4051,10 +4051,10 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SPD060</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="n">
+          <t>SPD0060</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="n">
         <v>21260</v>
       </c>
       <c r="C61" t="inlineStr">
@@ -4088,7 +4088,7 @@
           <t>Type 1</t>
         </is>
       </c>
-      <c r="J61" s="2" t="n">
+      <c r="J61" s="3" t="n">
         <v>45202</v>
       </c>
       <c r="K61" t="inlineStr">
@@ -4096,10 +4096,10 @@
           <t>Surgical</t>
         </is>
       </c>
-      <c r="L61" s="2" t="n">
+      <c r="L61" s="3" t="n">
         <v>45224</v>
       </c>
-      <c r="M61" s="2" t="n">
+      <c r="M61" s="3" t="n">
         <v>45887</v>
       </c>
       <c r="N61" t="inlineStr">

</xml_diff>

<commit_message>
edited bundled A3 form
</commit_message>
<xml_diff>
--- a/inst/extdata/a3_2025.xlsx
+++ b/inst/extdata/a3_2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ernestcaballero/Developer/data501/peridial/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA8AE699-BDE0-4245-B5F1-268D5DBA89BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72461883-9021-EF44-915C-A38FD1F87845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8740" yWindow="600" windowWidth="29660" windowHeight="19420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="116">
   <si>
     <t>Patient ID</t>
   </si>
@@ -362,6 +362,12 @@
   </si>
   <si>
     <t>Recurrent/Persistent Peritonitis</t>
+  </si>
+  <si>
+    <t>Transfer to HD</t>
+  </si>
+  <si>
+    <t>Transfer to hd</t>
   </si>
 </sst>
 </file>
@@ -2687,6 +2693,9 @@
       <c r="M47" s="3">
         <v>45981</v>
       </c>
+      <c r="N47" t="s">
+        <v>114</v>
+      </c>
       <c r="O47" t="s">
         <v>33</v>
       </c>
@@ -2736,6 +2745,9 @@
       </c>
       <c r="M48" s="3">
         <v>46021</v>
+      </c>
+      <c r="N48" t="s">
+        <v>115</v>
       </c>
       <c r="O48" t="s">
         <v>28</v>

</xml_diff>